<commit_message>
v3.3: refactor - spc pipeline(temp)
</commit_message>
<xml_diff>
--- a/resources/ctq_sheet_oos_decoration.xlsx
+++ b/resources/ctq_sheet_oos_decoration.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -53,9 +52,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -813,59 +813,6 @@
         <is>
           <t>flag</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ARRAY</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Z571</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1B990</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>RC_3</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>L3Z76700630</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="n">
-        <v>46223.489375</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.278268</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.087841</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.1111628166666667</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>USL</t>
-        </is>
-      </c>
-      <c r="M2" t="b">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>